<commit_message>
adding parrell exceution locally
</commit_message>
<xml_diff>
--- a/Daily_Tracker.xlsx
+++ b/Daily_Tracker.xlsx
@@ -1,32 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28925"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE5B6B06-A17A-4DCD-96AF-3B95D077C4AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456"/>
   </bookViews>
   <sheets>
-    <sheet name="TestResults" sheetId="1" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" r:id="rId2"/>
+    <sheet sheetId="1" name="TestResults" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Summary" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase">TestResults!$A$1:$A$1</definedName>
+    <definedName name="_xlnm._FilterDatabase">TestResults!$A$1</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="24">
   <si>
     <t>Test Case Title</t>
   </si>
   <si>
+    <t>02-08-2025</t>
+  </si>
+  <si>
     <t>01_Verify_Valid_Login</t>
   </si>
   <si>
+    <t>P</t>
+  </si>
+  <si>
     <t>02_Verify_Invalid_Login_by_wrong_password</t>
   </si>
   <si>
@@ -55,27 +60,75 @@
   </si>
   <si>
     <t>11_failed</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>SMK001_Verify user can log in with valid credentials</t>
+  </si>
+  <si>
+    <t>SMK002_Verify product list loads after login</t>
+  </si>
+  <si>
+    <t>SMK003_Verify user can add a product to cart</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Passed</t>
+  </si>
+  <si>
+    <t>Failed</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>% Passed</t>
+  </si>
+  <si>
+    <t>93%</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="006100"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="9C0006"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC7CE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -90,8 +143,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -431,169 +486,260 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A12"/>
-  <sheetFormatPr defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B15"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="58.5546875" customWidth="1"/>
     <col min="2" max="31" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" ht="14.4" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" ht="14.4" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+        <v>5</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+        <v>8</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>13</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:E1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:A28"/>
-  <sheetFormatPr defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E28"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="10.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25"/>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>13</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>14</v>
+      </c>
+      <c r="E2" t="s">
+        <v>23</v>
+      </c>
+    </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1"/>
-    </row>
-    <row r="5" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1"/>
-    </row>
-    <row r="6" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="1"/>
-    </row>
-    <row r="7" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="1"/>
-    </row>
-    <row r="8" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="1"/>
-    </row>
-    <row r="9" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="1"/>
-    </row>
-    <row r="10" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="1"/>
-    </row>
-    <row r="11" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="1"/>
-    </row>
-    <row r="12" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="1"/>
-    </row>
-    <row r="13" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="1"/>
-    </row>
-    <row r="14" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="1"/>
-    </row>
-    <row r="15" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="1"/>
-    </row>
-    <row r="16" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="1"/>
-    </row>
-    <row r="17" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="1"/>
-    </row>
-    <row r="18" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="1"/>
-    </row>
-    <row r="19" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="1"/>
-    </row>
-    <row r="20" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="1"/>
-    </row>
-    <row r="21" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="1"/>
-    </row>
-    <row r="22" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="1"/>
-    </row>
-    <row r="23" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="1"/>
-    </row>
-    <row r="24" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="1"/>
-    </row>
-    <row r="25" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="1"/>
-    </row>
-    <row r="26" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="1"/>
-    </row>
-    <row r="27" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="1"/>
-    </row>
-    <row r="28" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="1"/>
+      <c r="A4" s="3"/>
+    </row>
+    <row r="5" ht="14.4" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3"/>
+    </row>
+    <row r="6" ht="14.4" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" s="3"/>
+    </row>
+    <row r="7" ht="14.4" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3"/>
+    </row>
+    <row r="8" ht="14.4" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" s="3"/>
+    </row>
+    <row r="9" ht="14.4" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" s="3"/>
+    </row>
+    <row r="10" ht="14.4" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" s="3"/>
+    </row>
+    <row r="11" ht="14.4" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" s="3"/>
+    </row>
+    <row r="12" ht="14.4" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" s="3"/>
+    </row>
+    <row r="13" ht="14.4" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" s="3"/>
+    </row>
+    <row r="14" ht="14.4" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" s="3"/>
+    </row>
+    <row r="15" ht="14.4" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" s="3"/>
+    </row>
+    <row r="16" ht="14.4" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" s="3"/>
+    </row>
+    <row r="17" ht="14.4" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="3"/>
+    </row>
+    <row r="18" ht="14.4" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" s="3"/>
+    </row>
+    <row r="19" ht="14.4" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3"/>
+    </row>
+    <row r="20" ht="14.4" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3"/>
+    </row>
+    <row r="21" ht="14.4" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3"/>
+    </row>
+    <row r="22" ht="14.4" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3"/>
+    </row>
+    <row r="23" ht="14.4" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3"/>
+    </row>
+    <row r="24" ht="14.4" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3"/>
+    </row>
+    <row r="25" ht="14.4" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3"/>
+    </row>
+    <row r="26" ht="14.4" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" s="3"/>
+    </row>
+    <row r="27" ht="14.4" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" s="3"/>
+    </row>
+    <row r="28" ht="14.4" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
adding parrell test 1
</commit_message>
<xml_diff>
--- a/Daily_Tracker.xlsx
+++ b/Daily_Tracker.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="27">
   <si>
     <t>Test Case Title</t>
   </si>
@@ -74,6 +74,15 @@
     <t>SMK003_Verify user can add a product to cart</t>
   </si>
   <si>
+    <t>SMK001_Verify user can log in with valid credentials  @smoke</t>
+  </si>
+  <si>
+    <t>@smoke SMK002_Verify product list loads after login</t>
+  </si>
+  <si>
+    <t>@smoke SMK003_Verify user can add a product to cart</t>
+  </si>
+  <si>
     <t>Date</t>
   </si>
   <si>
@@ -89,7 +98,7 @@
     <t>% Passed</t>
   </si>
   <si>
-    <t>93%</t>
+    <t>94%</t>
   </si>
 </sst>
 </file>
@@ -487,7 +496,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="58.5546875" customWidth="1"/>
@@ -611,6 +620,30 @@
         <v>17</v>
       </c>
       <c r="B15" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -631,19 +664,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B1" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C1" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -651,16 +684,16 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>